<commit_message>
Version 30 OFFICIAL RELEASE
</commit_message>
<xml_diff>
--- a/outputs/Block2_First_Second_Exam_Progression_v12.xlsx
+++ b/outputs/Block2_First_Second_Exam_Progression_v12.xlsx
@@ -507,7 +507,7 @@
         <v>0.04824999999999999</v>
       </c>
       <c r="H2">
-        <v>0.02728243835797947</v>
+        <v>0.02728243835797942</v>
       </c>
       <c r="I2">
         <v>0.01891389104090235</v>
@@ -528,7 +528,7 @@
         <v>0.02795873786407774</v>
       </c>
       <c r="O2">
-        <v>0.006991176222057222</v>
+        <v>0.006991176222057166</v>
       </c>
       <c r="P2" t="b">
         <v>1</v>

</xml_diff>

<commit_message>
Visual Race Cards Publication
</commit_message>
<xml_diff>
--- a/outputs/Block2_First_Second_Exam_Progression_v12.xlsx
+++ b/outputs/Block2_First_Second_Exam_Progression_v12.xlsx
@@ -507,7 +507,7 @@
         <v>0.04824999999999999</v>
       </c>
       <c r="H2">
-        <v>0.02728243835797947</v>
+        <v>0.02728243835797942</v>
       </c>
       <c r="I2">
         <v>0.01891389104090235</v>
@@ -528,7 +528,7 @@
         <v>0.02795873786407774</v>
       </c>
       <c r="O2">
-        <v>0.006991176222057222</v>
+        <v>0.006991176222057166</v>
       </c>
       <c r="P2" t="b">
         <v>1</v>
@@ -719,7 +719,7 @@
         <v>0.01862500000000003</v>
       </c>
       <c r="H6">
-        <v>0.002187908649066761</v>
+        <v>0.002187908649066789</v>
       </c>
       <c r="I6">
         <v>0.005372069085689518</v>
@@ -740,7 +740,7 @@
         <v>0.0172500000000001</v>
       </c>
       <c r="O6">
-        <v>0.0008129086490668291</v>
+        <v>0.0008129086490668569</v>
       </c>
       <c r="P6" t="b">
         <v>1</v>

</xml_diff>